<commit_message>
Terminat Verificare Defecte Cod + Refactorizare
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Laptop\e\VVSS\CamiVVSS_ro2025-2026\Labs\CheckListsAll\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Facultate\VVSS\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE83867-3721-469D-B0A3-67FDA22FF09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69D8F9F-0006-455A-A4AE-EC998CD3C0AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="72">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -135,13 +135,135 @@
   </si>
   <si>
     <t>Effort to perform tool-based code analysis (hours):</t>
+  </si>
+  <si>
+    <t>Secure George-Sebastian</t>
+  </si>
+  <si>
+    <t>Stanca Vlad Tudor</t>
+  </si>
+  <si>
+    <t>C01</t>
+  </si>
+  <si>
+    <t>C04</t>
+  </si>
+  <si>
+    <t>C06</t>
+  </si>
+  <si>
+    <t>C07</t>
+  </si>
+  <si>
+    <t>C08</t>
+  </si>
+  <si>
+    <t>C09</t>
+  </si>
+  <si>
+    <t>Prelucrarea datelor trebuie făcută în service/repository, nu în controller</t>
+  </si>
+  <si>
+    <t>DrinkShopApp 21-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DrinkShopApp </t>
+  </si>
+  <si>
+    <t>Nu se gestionează erorile - "throws Exception"</t>
+  </si>
+  <si>
+    <t>Prelucrările (filtrările) ar trebui realizare în repository</t>
+  </si>
+  <si>
+    <t>ProductService 45, 52</t>
+  </si>
+  <si>
+    <t>La update se inserează toți parametri obiectului în loc de o instanța lui (=&gt; updateProduct(prod) )</t>
+  </si>
+  <si>
+    <t>Toate Service-urile</t>
+  </si>
+  <si>
+    <t>La metodele de Add și Update nu sunt apelați validatorii</t>
+  </si>
+  <si>
+    <t>ProductService 21
+DrinkShopService 38</t>
+  </si>
+  <si>
+    <t>DrinkShopService 23</t>
+  </si>
+  <si>
+    <t>Repository&lt;Integer,Stoc&gt; stocService =&gt; stocRepo</t>
+  </si>
+  <si>
+    <t>C12</t>
+  </si>
+  <si>
+    <t>RetetaValidator 14</t>
+  </si>
+  <si>
+    <t>Tipul declarat este double, însă se pune ca parametru int</t>
+  </si>
+  <si>
+    <t>FileStocRepository 24-27
+Stoc 10</t>
+  </si>
+  <si>
+    <t>.get(0) poate arunca IndexOutOfBoundsException</t>
+  </si>
+  <si>
+    <t>ReceiptGenerator
+CsvExporter</t>
+  </si>
+  <si>
+    <t>C11</t>
+  </si>
+  <si>
+    <t>Repository-uri</t>
+  </si>
+  <si>
+    <t>Service-uri/Repository-uri</t>
+  </si>
+  <si>
+    <t>Nu se verifică dacă operațiile din fișiere se execută corect - nu se gestionează erorile IO. Nu se verifică existența duplicatelor</t>
+  </si>
+  <si>
+    <t>DrinkShopController</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Există metoda ShowError pentru erori, dar nu există și pentru warnings, infos - cod duplicat </t>
+  </si>
+  <si>
+    <t>OrderService 43
+DrinkShopController 123</t>
+  </si>
+  <si>
+    <t>Metodă ineficientă - există deja implementare a metodei utilizate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OrderService 43
+</t>
+  </si>
+  <si>
+    <t>Nu se verifică dacă repository-urile sunt create corect. Problemă ce apare din cauza căilor relative ale fișierelor -</t>
+  </si>
+  <si>
+    <t>Nu se verifică dacă datele de intrare sunt valide în metoda extractEntity</t>
+  </si>
+  <si>
+    <t>De ce se folosește AtomicReference și nu String/StringBuilder?</t>
+  </si>
+  <si>
+    <t>Metodă ineficientă. Poți lua Product din OrderItem și nu prin stream</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -224,6 +346,15 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -326,7 +457,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -398,6 +529,31 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -707,19 +863,19 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.26953125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.453125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.90625" style="6"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="4" width="16.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.85546875" style="6"/>
     <col min="9" max="9" width="21" style="6" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.90625" style="6"/>
+    <col min="10" max="10" width="14.42578125" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -730,7 +886,7 @@
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
         <v>19</v>
       </c>
@@ -745,14 +901,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
       <c r="I3" s="17"/>
       <c r="J3" s="17"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
@@ -766,7 +922,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
@@ -780,7 +936,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
@@ -788,14 +944,14 @@
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -809,7 +965,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -817,7 +973,7 @@
       <c r="D10" s="1"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -826,7 +982,7 @@
       <c r="D11" s="1"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
@@ -835,7 +991,7 @@
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -844,7 +1000,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -853,7 +1009,7 @@
       <c r="D14" s="1"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -862,7 +1018,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -871,7 +1027,7 @@
       <c r="D16" s="1"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -880,7 +1036,7 @@
       <c r="D17" s="1"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -889,7 +1045,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="15"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -898,7 +1054,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="15"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -907,7 +1063,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -916,7 +1072,7 @@
       <c r="D21" s="3"/>
       <c r="E21" s="15"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -925,7 +1081,7 @@
       <c r="D22" s="3"/>
       <c r="E22" s="15"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -934,7 +1090,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="15"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -943,7 +1099,7 @@
       <c r="D24" s="3"/>
       <c r="E24" s="15"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -952,7 +1108,7 @@
       <c r="D25" s="3"/>
       <c r="E25" s="15"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C27" s="11" t="s">
         <v>8</v>
       </c>
@@ -979,18 +1135,18 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.26953125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.453125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.90625" style="6"/>
-    <col min="9" max="9" width="22.08984375" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.90625" style="6"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="4" width="16.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.85546875" style="6"/>
+    <col min="9" max="9" width="22.140625" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -1001,7 +1157,7 @@
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
         <v>18</v>
       </c>
@@ -1016,14 +1172,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
       <c r="I3" s="17"/>
       <c r="J3" s="17"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
@@ -1037,7 +1193,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
@@ -1051,7 +1207,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
@@ -1059,14 +1215,14 @@
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1080,7 +1236,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1088,7 +1244,7 @@
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1097,7 +1253,7 @@
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B26" si="0">B11+1</f>
         <v>3</v>
@@ -1106,7 +1262,7 @@
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1115,7 +1271,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1124,7 +1280,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1133,7 +1289,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1142,7 +1298,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1151,7 +1307,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1160,7 +1316,7 @@
       <c r="D18" s="1"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1169,7 +1325,7 @@
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1178,7 +1334,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1187,7 +1343,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1196,7 +1352,7 @@
       <c r="D22" s="1"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1205,7 +1361,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1214,7 +1370,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1223,7 +1379,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1232,7 +1388,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C28" s="11" t="s">
         <v>8</v>
       </c>
@@ -1258,20 +1414,21 @@
   <sheetPr>
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.26953125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.453125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.90625" style="6"/>
-    <col min="9" max="9" width="26.7265625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.90625" style="6"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="22.5703125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="51.7109375" style="6" customWidth="1"/>
+    <col min="6" max="7" width="8.85546875" style="6"/>
+    <col min="8" max="8" width="11.140625" style="6" customWidth="1"/>
+    <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -1282,7 +1439,7 @@
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
         <v>17</v>
       </c>
@@ -1297,14 +1454,18 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I3" s="38" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" s="37">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
@@ -1315,10 +1476,14 @@
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I4" s="39" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="37">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
@@ -1332,22 +1497,26 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22"/>
+      <c r="D6" s="22" t="s">
+        <v>33</v>
+      </c>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22"/>
+      <c r="D7" s="36">
+        <v>46091</v>
+      </c>
       <c r="E7" s="22"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1361,200 +1530,280 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B10" s="3">
+    <row r="10" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="44">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B11" s="3">
-        <f>B10+1</f>
+      <c r="C10" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="43" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="B11" s="44">
+        <f t="shared" ref="B11:B24" si="0">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B12" s="3">
-        <f t="shared" ref="B12:B30" si="0">B11+1</f>
+      <c r="C11" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="41" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="42" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B12" s="44">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B13" s="3">
+      <c r="C12" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="41" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="42" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B13" s="44">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B14" s="3">
+      <c r="C13" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="43" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B14" s="44">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B15" s="3">
+      <c r="C14" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="41" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B15" s="44">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B16" s="3">
+      <c r="C15" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="41" t="s">
+        <v>67</v>
+      </c>
+      <c r="E15" s="43" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B16" s="44">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B17" s="3">
+      <c r="C16" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="41" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" s="43" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="44">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B18" s="3">
+      <c r="C17" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="41" t="s">
+        <v>48</v>
+      </c>
+      <c r="E17" s="43" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="B18" s="44">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B19" s="3">
+      <c r="C18" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" s="43" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="B19" s="44">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B20" s="3">
+      <c r="C19" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="41" t="s">
+        <v>58</v>
+      </c>
+      <c r="E19" s="43" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="B20" s="44">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="1"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B21" s="3">
+      <c r="C20" s="40" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" s="41" t="s">
+        <v>61</v>
+      </c>
+      <c r="E20" s="43" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="44">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="2"/>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B22" s="3">
+      <c r="C21" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="E21" s="43" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="B22" s="44">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="1"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B23" s="3">
+      <c r="C22" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" s="41" t="s">
+        <v>50</v>
+      </c>
+      <c r="E22" s="43" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B23" s="44">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="1"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B24" s="3">
+      <c r="C23" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="D23" s="41" t="s">
+        <v>51</v>
+      </c>
+      <c r="E23" s="43" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="B24" s="44">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="1"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B25" s="3">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="C25" s="1"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B26" s="3">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="2"/>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B27" s="3">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="C27" s="1"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="1"/>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B28" s="3">
-        <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-      <c r="C28" s="1"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B29" s="3">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="C29" s="1"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B30" s="3">
-        <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-      <c r="C30" s="1"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-    </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="C32" s="11" t="s">
+      <c r="C24" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="D24" s="41" t="s">
+        <v>56</v>
+      </c>
+      <c r="E24" s="43" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="3"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="43"/>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="3"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="43"/>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="3"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="43"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="3"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="43"/>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="3"/>
+      <c r="C29" s="40"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="43"/>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="3"/>
+      <c r="C30" s="40"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="43"/>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="3"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="43"/>
+    </row>
+    <row r="33" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C33" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D32" s="12"/>
-      <c r="E32" s="1"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="1">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1576,20 +1825,20 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.26953125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.90625" style="6" customWidth="1"/>
-    <col min="6" max="6" width="16.6328125" style="6" customWidth="1"/>
-    <col min="7" max="8" width="8.90625" style="6"/>
-    <col min="9" max="9" width="26.7265625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.90625" style="6"/>
+    <col min="5" max="5" width="23.85546875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="6" customWidth="1"/>
+    <col min="7" max="8" width="8.85546875" style="6"/>
+    <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
@@ -1600,7 +1849,7 @@
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
         <v>31</v>
       </c>
@@ -1615,14 +1864,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
       <c r="I3" s="17"/>
       <c r="J3" s="17"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
@@ -1634,7 +1883,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
@@ -1646,7 +1895,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>1</v>
@@ -1655,7 +1904,7 @@
       <c r="E6" s="22"/>
       <c r="F6" s="20"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1672,7 +1921,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1681,7 +1930,7 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1691,7 +1940,7 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
@@ -1701,7 +1950,7 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1711,7 +1960,7 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1721,7 +1970,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1731,7 +1980,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1741,7 +1990,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1751,7 +2000,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1761,7 +2010,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1771,7 +2020,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1781,7 +2030,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1791,7 +2040,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1801,7 +2050,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1811,7 +2060,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1821,7 +2070,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1831,7 +2080,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1841,7 +2090,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1851,7 +2100,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1861,7 +2110,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1871,7 +2120,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1881,7 +2130,7 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C32" s="34" t="s">
         <v>32</v>
       </c>
@@ -1889,7 +2138,7 @@
       <c r="E32" s="35"/>
       <c r="F32" s="18"/>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F35" s="21"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
commit completare tabel requirements
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Informatica\vvss\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB49BF7-55C4-4CF1-9C70-7E0952C11976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3C91FCB-176C-4B1B-AA39-2209B260BE44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -287,7 +287,7 @@
     <t>30 min</t>
   </si>
   <si>
-    <t xml:space="preserve">La finalul unei zile nu este specificat cum se salveaza </t>
+    <t>La finalul unei zile nu este specificat modul de salvare a informatiilor despre comenzile inregistrate: manual sau automat</t>
   </si>
 </sst>
 </file>
@@ -540,6 +540,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="16" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -549,43 +550,42 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="16" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -912,11 +912,11 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
@@ -948,10 +948,10 @@
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="36"/>
+      <c r="E4" s="34"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -966,10 +966,10 @@
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="37" t="s">
+      <c r="D5" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="38"/>
+      <c r="E5" s="36"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -981,19 +981,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="31"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="29">
+      <c r="D7" s="30">
         <v>46091</v>
       </c>
-      <c r="E7" s="30"/>
+      <c r="E7" s="31"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -1062,7 +1062,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1179,7 +1179,7 @@
         <v>8</v>
       </c>
       <c r="D27" s="12"/>
-      <c r="E27" s="44" t="s">
+      <c r="E27" s="29" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1219,11 +1219,11 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
@@ -1255,10 +1255,10 @@
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="39" t="s">
+      <c r="D4" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="39"/>
+      <c r="E4" s="37"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1273,10 +1273,10 @@
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="41"/>
+      <c r="E5" s="39"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1288,19 +1288,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="31"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="29">
+      <c r="D7" s="30">
         <v>46091</v>
       </c>
-      <c r="E7" s="30"/>
+      <c r="E7" s="31"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -1513,11 +1513,11 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
@@ -1549,10 +1549,10 @@
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="32"/>
+      <c r="E4" s="40"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1567,10 +1567,10 @@
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="35"/>
+      <c r="E5" s="42"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1582,19 +1582,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="31"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="29">
+      <c r="D7" s="30">
         <v>46091</v>
       </c>
-      <c r="E7" s="30"/>
+      <c r="E7" s="31"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -1923,11 +1923,11 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
@@ -1955,8 +1955,8 @@
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1967,8 +1967,8 @@
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1980,8 +1980,8 @@
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
       <c r="F6" s="20"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -2211,11 +2211,11 @@
       <c r="F30" s="2"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C32" s="42" t="s">
+      <c r="C32" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="43"/>
-      <c r="E32" s="43"/>
+      <c r="D32" s="44"/>
+      <c r="E32" s="44"/>
       <c r="F32" s="18"/>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
commit completare tabel arhitectura
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Informatica\vvss\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3C91FCB-176C-4B1B-AA39-2209B260BE44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5787AE9A-AC2E-4E64-BA4E-671A252658C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="92">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -288,6 +288,33 @@
   </si>
   <si>
     <t>La finalul unei zile nu este specificat modul de salvare a informatiilor despre comenzile inregistrate: manual sau automat</t>
+  </si>
+  <si>
+    <t>A01</t>
+  </si>
+  <si>
+    <t>A03</t>
+  </si>
+  <si>
+    <t>A05</t>
+  </si>
+  <si>
+    <t>Requirements_MyDrinkShop.ong</t>
+  </si>
+  <si>
+    <t>DrinkShopService primeste in constructor repository-uri, cand el ar trebui sa primeasca service-urile create din exterior, conform Dependency Injection</t>
+  </si>
+  <si>
+    <t>A10</t>
+  </si>
+  <si>
+    <t>Nu exista nicio legatura intre reteta si produse, o reteta ar trebui sa tina de / sa depinda de un produs existent</t>
+  </si>
+  <si>
+    <t>Nu este clar din diagrama care este legatura validatorilor cu restul claselor din proiect</t>
+  </si>
+  <si>
+    <t>Nu este deloc clar, lipseste implementarea functionalitatii 3, cea de adaugare, modificare si stergere a tipului si categoriei de bautura</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1234,8 @@
   <cols>
     <col min="1" max="1" width="8.85546875" style="6"/>
     <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
     <col min="6" max="8" width="8.85546875" style="6"/>
     <col min="9" max="9" width="22.140625" style="6" customWidth="1"/>
@@ -1316,40 +1344,58 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C10" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E11" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B26" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>85</v>
+      </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E12" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>84</v>
+      </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="2"/>
+      <c r="E13" s="2" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
@@ -1473,7 +1519,9 @@
         <v>8</v>
       </c>
       <c r="D28" s="12"/>
-      <c r="E28" s="1"/>
+      <c r="E28" s="1">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
Terminat Verificare Folosind SonarQube
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Informatica\vvss\docs\Lab01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Facultate\VVSS\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5787AE9A-AC2E-4E64-BA4E-671A252658C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7D790E4-A94E-418E-A709-49B0F3858C03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="650" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="650" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="122">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -315,13 +315,114 @@
   </si>
   <si>
     <t>Nu este deloc clar, lipseste implementarea functionalitatii 3, cea de adaugare, modificare si stergere a tipului si categoriei de bautura</t>
+  </si>
+  <si>
+    <t>SonarQube</t>
+  </si>
+  <si>
+    <t>CsvExporter 14</t>
+  </si>
+  <si>
+    <t>"Add a private constructor to hide the implicit public one"</t>
+  </si>
+  <si>
+    <t>CsvExporter 20</t>
+  </si>
+  <si>
+    <t>class CsvExporter { // Noncompliant
+…
+}</t>
+  </si>
+  <si>
+    <t>class CsvExporter { // Compliant
+  private CsvExporter() {
+    /* This utility class should not be instantiated */
+  }</t>
+  </si>
+  <si>
+    <t>public static void exportOrders(List&lt;Product&gt; products, List&lt;Order&gt; orders, String path)</t>
+  </si>
+  <si>
+    <t>public static void exportOrders(List&lt;Order&gt; orders, String path)</t>
+  </si>
+  <si>
+    <t>CsvExporter 39</t>
+  </si>
+  <si>
+    <t>catch (IOException e) {
+            throw new RuntimeException(e);
+        }</t>
+  </si>
+  <si>
+    <t>catch (IOException e) {
+            throw new CsvExportException(e);
+        }</t>
+  </si>
+  <si>
+    <t>FileAbstractRepository 12</t>
+  </si>
+  <si>
+    <t>public FileAbstractRepository(String fileName)</t>
+  </si>
+  <si>
+    <t>protected FileAbstractRepository(String fileName)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> //loadFromFile();</t>
+  </si>
+  <si>
+    <t>FileAbstractRepository 14</t>
+  </si>
+  <si>
+    <t>FileAbstractRepository 7</t>
+  </si>
+  <si>
+    <t>"Unused method parameters should be removed"</t>
+  </si>
+  <si>
+    <t>"Generic exceptions should never be thrown"</t>
+  </si>
+  <si>
+    <t>"Constructors of an "abstract" class should not be declared "public""</t>
+  </si>
+  <si>
+    <t>"Sections of code should not be commented out"</t>
+  </si>
+  <si>
+    <t>"Type parameter names should comply with a naming convention"</t>
+  </si>
+  <si>
+    <t>"ID" este mai ușor de înțeles, decât doar "I"</t>
+  </si>
+  <si>
+    <t>"Lambdas containing only one statement should not nest this statement in a block"</t>
+  </si>
+  <si>
+    <t>RetetaValidator 27-29</t>
+  </si>
+  <si>
+    <t>.forEach(entry -&gt; {          errors.append("[").append(entry.getDenumire()).append("]").append("cantitate negativa sau zero").append("\n");
+                });</t>
+  </si>
+  <si>
+    <t>.forEach(entry -&gt;
+errors.append("[").append(entry.getDenumire()).append("]").append("cantitate negativa sau zero").append("\n"));</t>
+  </si>
+  <si>
+    <t>"Unused "private" fields should be removed"</t>
+  </si>
+  <si>
+    <t>OrderService 14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    private final Repository&lt;Integer, Product&gt; productRepo;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -414,6 +515,14 @@
       <family val="2"/>
       <charset val="238"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+      <charset val="238"/>
     </font>
   </fonts>
   <fills count="5">
@@ -515,7 +624,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -568,17 +677,26 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -589,15 +707,6 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -612,6 +721,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -939,19 +1051,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="H1" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -975,10 +1087,10 @@
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="D4" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="34"/>
+      <c r="E4" s="37"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -993,10 +1105,10 @@
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="35" t="s">
+      <c r="D5" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="36"/>
+      <c r="E5" s="39"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1008,19 +1120,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="31"/>
+      <c r="E6" s="33"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="30">
+      <c r="D7" s="34">
         <v>46091</v>
       </c>
-      <c r="E7" s="31"/>
+      <c r="E7" s="33"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -1247,19 +1359,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="H1" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1283,10 +1395,10 @@
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="37"/>
+      <c r="E4" s="32"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
@@ -1301,10 +1413,10 @@
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="39"/>
+      <c r="E5" s="36"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -1316,19 +1428,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="31"/>
+      <c r="E6" s="33"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="30">
+      <c r="D7" s="34">
         <v>46091</v>
       </c>
-      <c r="E7" s="31"/>
+      <c r="E7" s="33"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -1561,19 +1673,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="H1" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1630,19 +1742,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="31"/>
+      <c r="E6" s="33"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="30">
+      <c r="D7" s="34">
         <v>46091</v>
       </c>
-      <c r="E7" s="31"/>
+      <c r="E7" s="33"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -1957,10 +2069,10 @@
   <cols>
     <col min="1" max="1" width="8.85546875" style="6"/>
     <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
-    <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.85546875" style="6" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="23.5703125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="49" style="6" customWidth="1"/>
+    <col min="5" max="5" width="48.85546875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="52.140625" style="6" customWidth="1"/>
     <col min="7" max="8" width="8.85546875" style="6"/>
     <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
     <col min="10" max="16384" width="8.85546875" style="6"/>
@@ -1971,19 +2083,19 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="H1" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1996,27 +2108,39 @@
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
+      <c r="I3" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" s="9">
+        <v>236</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="40"/>
+      <c r="D4" s="40" t="s">
+        <v>92</v>
+      </c>
       <c r="E4" s="40"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="I4" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="9">
+        <v>236</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
+      <c r="D5" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="33"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
@@ -2028,8 +2152,10 @@
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
+      <c r="D6" s="34">
+        <v>46092</v>
+      </c>
+      <c r="E6" s="33"/>
       <c r="F6" s="20"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -2049,174 +2175,232 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C10" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="E10" s="45" t="s">
+        <v>96</v>
+      </c>
+      <c r="F10" s="45" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C11" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="E11" s="45" t="s">
+        <v>98</v>
+      </c>
+      <c r="F11" s="45" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="36" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C12" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="E12" s="45" t="s">
+        <v>101</v>
+      </c>
+      <c r="F12" s="45" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+      <c r="C13" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="E13" s="45" t="s">
+        <v>104</v>
+      </c>
+      <c r="F13" s="45" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C14" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="D14" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" s="45" t="s">
+        <v>106</v>
+      </c>
+      <c r="F14" s="45"/>
+    </row>
+    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C15" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="E15" s="45"/>
+      <c r="F15" s="45" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C16" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="E16" s="45" t="s">
+        <v>117</v>
+      </c>
+      <c r="F16" s="45" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="24" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
+      <c r="C17" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="E17" s="45" t="s">
+        <v>121</v>
+      </c>
+      <c r="F17" s="45"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="45"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="45"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="1"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="45"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="45"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="1"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="1"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="1"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="1"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="3">

</xml_diff>